<commit_message>
error check for empty column
</commit_message>
<xml_diff>
--- a/293810_I.xlsx
+++ b/293810_I.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lucas\TreadStone\testing\293810_I\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lucas\TreadStone\label-maker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A79EA1B-4668-4FE5-831F-F5C1339606E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550FF6BA-E732-4278-BF89-812B166B20D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="38">
   <si>
     <t>Batch</t>
   </si>
@@ -145,26 +145,20 @@
     <t>mΩ*cm2</t>
   </si>
   <si>
-    <t>24103R1</t>
-  </si>
-  <si>
-    <t>240718-I</t>
-  </si>
-  <si>
     <t>M38</t>
   </si>
   <si>
     <t>1110-038-2</t>
   </si>
   <si>
-    <t>293810_I</t>
+    <t>260214_I</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -206,14 +200,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -223,7 +209,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -263,21 +249,6 @@
         <color rgb="FFCCCCCC"/>
       </right>
       <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
         <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
@@ -289,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -321,15 +292,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -665,7 +627,7 @@
         <v>20</v>
       </c>
       <c r="B1" s="18">
-        <v>293810</v>
+        <v>26024</v>
       </c>
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
@@ -685,23 +647,13 @@
       <c r="R1" s="16"/>
       <c r="S1" s="16"/>
       <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="16"/>
-      <c r="Y1" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="Z1" s="16" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="2" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -721,16 +673,6 @@
       <c r="R2" s="16"/>
       <c r="S2" s="16"/>
       <c r="T2" s="16"/>
-      <c r="U2" s="16"/>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="X2" s="16"/>
-      <c r="Y2" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="16" t="s">
-        <v>36</v>
-      </c>
     </row>
     <row r="3" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="17" t="s">
@@ -757,24 +699,15 @@
       <c r="R3" s="16"/>
       <c r="S3" s="16"/>
       <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="17" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z3" s="19">
-        <v>45491</v>
-      </c>
+      <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:41" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
     </row>
-    <row r="6" spans="1:41" s="8" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:41" s="8" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
@@ -809,13 +742,13 @@
       <c r="AF6" s="9"/>
       <c r="AG6" s="9"/>
       <c r="AI6" s="9"/>
-      <c r="AK6" s="17"/>
-      <c r="AL6" s="16"/>
-      <c r="AM6" s="16"/>
-      <c r="AN6" s="17"/>
-      <c r="AO6" s="16"/>
-    </row>
-    <row r="7" spans="1:41" s="8" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="AK6"/>
+      <c r="AL6"/>
+      <c r="AM6"/>
+      <c r="AN6"/>
+      <c r="AO6"/>
+    </row>
+    <row r="7" spans="1:41" s="8" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>2</v>
       </c>
@@ -865,1467 +798,1084 @@
         <v>12</v>
       </c>
       <c r="U7" s="10"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="11"/>
-      <c r="X7" s="10"/>
-      <c r="Y7" s="10"/>
-      <c r="Z7" s="11"/>
-      <c r="AA7" s="10"/>
-      <c r="AB7" s="10"/>
-      <c r="AC7" s="11"/>
-      <c r="AD7" s="10"/>
-      <c r="AE7" s="10"/>
-      <c r="AF7" s="11"/>
-      <c r="AG7" s="11"/>
-      <c r="AH7" s="10"/>
-      <c r="AI7" s="11"/>
-      <c r="AK7" s="21"/>
-      <c r="AL7" s="21"/>
-      <c r="AM7" s="20"/>
-      <c r="AN7" s="21"/>
-      <c r="AO7" s="21"/>
-    </row>
-    <row r="8" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="V7"/>
+      <c r="W7"/>
+      <c r="X7"/>
+      <c r="Y7"/>
+      <c r="Z7"/>
+      <c r="AA7"/>
+      <c r="AB7"/>
+      <c r="AC7"/>
+      <c r="AD7"/>
+      <c r="AE7"/>
+      <c r="AF7"/>
+      <c r="AG7"/>
+      <c r="AH7"/>
+      <c r="AI7"/>
+      <c r="AJ7"/>
+      <c r="AK7"/>
+      <c r="AL7"/>
+      <c r="AM7"/>
+      <c r="AN7"/>
+      <c r="AO7"/>
+    </row>
+    <row r="8" spans="1:41" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" s="1">
         <v>1498</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E8" s="1">
         <v>1528</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H8" s="1">
         <v>1477</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K8" s="1">
         <v>1340</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N8" s="1">
         <v>1101</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q8" s="1">
         <v>1091</v>
       </c>
       <c r="S8" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T8" s="1">
         <v>1339</v>
       </c>
-      <c r="V8" s="1"/>
-      <c r="W8" s="1"/>
-      <c r="Y8" s="1"/>
-      <c r="Z8" s="1"/>
-      <c r="AB8" s="1"/>
-      <c r="AC8" s="1"/>
-      <c r="AE8" s="1"/>
-      <c r="AF8" s="1"/>
-      <c r="AG8" s="6"/>
-      <c r="AH8" s="1"/>
-      <c r="AI8" s="1"/>
-      <c r="AK8" s="17"/>
-      <c r="AL8" s="22"/>
-      <c r="AM8" s="16"/>
-      <c r="AN8" s="17"/>
-      <c r="AO8" s="18"/>
-    </row>
-    <row r="9" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1">
         <v>1615</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E9" s="1">
         <v>780</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H9" s="1">
         <v>1428</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K9" s="1">
         <v>1311</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N9" s="1">
         <v>1365</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q9" s="1">
         <v>1259</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T9" s="1">
         <v>1337</v>
       </c>
-      <c r="V9" s="1"/>
-      <c r="W9" s="1"/>
-      <c r="Y9" s="1"/>
-      <c r="Z9" s="1"/>
-      <c r="AB9" s="1"/>
-      <c r="AC9" s="1"/>
-      <c r="AE9" s="1"/>
-      <c r="AF9" s="1"/>
-      <c r="AG9" s="6"/>
-      <c r="AH9" s="1"/>
-      <c r="AI9" s="1"/>
-      <c r="AK9" s="17"/>
-      <c r="AL9" s="18"/>
-      <c r="AM9" s="16"/>
-      <c r="AN9" s="17"/>
-      <c r="AO9" s="18"/>
-    </row>
-    <row r="10" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B10" s="1">
         <v>1603</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E10" s="1">
         <v>1049</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H10" s="1">
         <v>1284</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K10" s="1">
         <v>1316</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N10" s="1">
         <v>1081</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q10" s="1">
         <v>1296</v>
       </c>
       <c r="S10" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T10" s="1">
         <v>1066</v>
       </c>
-      <c r="V10" s="1"/>
-      <c r="W10" s="1"/>
-      <c r="Y10" s="1"/>
-      <c r="Z10" s="1"/>
-      <c r="AB10" s="1"/>
-      <c r="AC10" s="1"/>
-      <c r="AE10" s="1"/>
-      <c r="AF10" s="1"/>
-      <c r="AG10" s="6"/>
-      <c r="AH10" s="1"/>
-      <c r="AI10" s="1"/>
-      <c r="AK10" s="17"/>
-      <c r="AL10" s="18"/>
-      <c r="AM10" s="16"/>
-      <c r="AN10" s="17"/>
-      <c r="AO10" s="18"/>
-    </row>
-    <row r="11" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="11" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1">
         <v>1444</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E11" s="1">
         <v>1499</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H11" s="1">
         <v>1425</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K11" s="1">
         <v>1127</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N11" s="1">
         <v>1343</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q11">
         <v>1063</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T11" s="1">
         <v>1082</v>
       </c>
-      <c r="V11" s="1"/>
-      <c r="W11" s="1"/>
-      <c r="Y11" s="1"/>
-      <c r="Z11" s="1"/>
-      <c r="AB11" s="1"/>
-      <c r="AC11" s="1"/>
-      <c r="AE11" s="1"/>
-      <c r="AF11" s="1"/>
-      <c r="AG11" s="6"/>
-      <c r="AH11" s="1"/>
-      <c r="AI11" s="1"/>
-      <c r="AK11" s="17"/>
-      <c r="AL11" s="18"/>
-      <c r="AM11" s="16"/>
-      <c r="AN11" s="17"/>
-      <c r="AO11" s="18"/>
-    </row>
-    <row r="12" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B12" s="1">
         <v>1616</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E12" s="1">
         <v>778</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H12" s="1">
         <v>1393</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K12" s="1">
         <v>1196</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N12" s="1">
         <v>1278</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q12" s="1">
         <v>1329</v>
       </c>
       <c r="S12" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T12" s="1">
         <v>1375</v>
       </c>
-      <c r="V12" s="1"/>
-      <c r="W12" s="1"/>
-      <c r="Y12" s="1"/>
-      <c r="Z12" s="1"/>
-      <c r="AB12" s="1"/>
-      <c r="AC12" s="1"/>
-      <c r="AE12" s="1"/>
-      <c r="AF12" s="1"/>
-      <c r="AG12" s="6"/>
-      <c r="AH12" s="1"/>
-      <c r="AI12" s="1"/>
-      <c r="AK12" s="17"/>
-      <c r="AL12" s="18"/>
-      <c r="AM12" s="16"/>
-      <c r="AN12" s="17"/>
-      <c r="AO12" s="18"/>
-    </row>
-    <row r="13" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B13" s="1">
         <v>1601</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E13">
         <v>1582</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H13" s="1">
         <v>1410</v>
       </c>
       <c r="J13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K13">
         <v>1266</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N13" s="1">
         <v>1273</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q13">
         <v>1056</v>
       </c>
       <c r="S13" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T13" s="1">
         <v>1226</v>
       </c>
-      <c r="V13" s="1"/>
-      <c r="W13" s="1"/>
-      <c r="Y13" s="1"/>
-      <c r="Z13" s="1"/>
-      <c r="AB13" s="1"/>
-      <c r="AC13" s="1"/>
-      <c r="AE13" s="1"/>
-      <c r="AF13" s="1"/>
-      <c r="AG13" s="6"/>
-      <c r="AH13" s="1"/>
-      <c r="AI13" s="1"/>
-      <c r="AK13" s="17"/>
-      <c r="AL13" s="18"/>
-      <c r="AM13" s="16"/>
-      <c r="AN13" s="17"/>
-      <c r="AO13" s="18"/>
-    </row>
-    <row r="14" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="14" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B14" s="1">
         <v>1617</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E14">
         <v>1544</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H14" s="1">
         <v>1443</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K14" s="1">
         <v>1210</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N14" s="1">
         <v>1215</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q14" s="1">
         <v>1241</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T14" s="1">
         <v>1300</v>
       </c>
-      <c r="V14" s="1"/>
-      <c r="W14" s="1"/>
-      <c r="Y14" s="1"/>
-      <c r="Z14" s="1"/>
-      <c r="AB14" s="1"/>
-      <c r="AC14" s="1"/>
-      <c r="AE14" s="1"/>
-      <c r="AF14" s="1"/>
-      <c r="AG14" s="6"/>
-      <c r="AH14" s="1"/>
-      <c r="AI14" s="1"/>
-      <c r="AK14" s="17"/>
-      <c r="AL14" s="18"/>
-      <c r="AM14" s="16"/>
-      <c r="AN14" s="17"/>
-      <c r="AO14" s="18"/>
-    </row>
-    <row r="15" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="15" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B15" s="1">
         <v>1566</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E15">
         <v>1495</v>
       </c>
       <c r="G15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H15" s="1">
         <v>1189</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K15" s="1">
         <v>1294</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N15" s="1">
         <v>1324</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q15">
         <v>1263</v>
       </c>
       <c r="S15" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T15" s="1">
         <v>1326</v>
       </c>
-      <c r="V15" s="1"/>
-      <c r="W15" s="1"/>
-      <c r="Y15" s="1"/>
-      <c r="Z15" s="1"/>
-      <c r="AB15" s="1"/>
-      <c r="AC15" s="1"/>
-      <c r="AE15" s="1"/>
-      <c r="AF15" s="1"/>
-      <c r="AG15" s="6"/>
-      <c r="AH15" s="1"/>
-      <c r="AI15" s="1"/>
-      <c r="AK15" s="17"/>
-      <c r="AL15" s="18"/>
-      <c r="AM15" s="16"/>
-      <c r="AN15" s="17"/>
-      <c r="AO15" s="18"/>
-    </row>
-    <row r="16" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="1:41" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B16" s="1">
         <v>1568</v>
       </c>
       <c r="D16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E16">
         <v>1491</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H16" s="1">
         <v>1567</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K16" s="1">
         <v>1335</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N16" s="1">
         <v>1090</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q16" s="1">
         <v>1321</v>
       </c>
       <c r="S16" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T16" s="1">
         <v>1275</v>
       </c>
-      <c r="V16" s="1"/>
-      <c r="W16" s="1"/>
-      <c r="Y16" s="1"/>
-      <c r="Z16" s="1"/>
-      <c r="AB16" s="1"/>
-      <c r="AC16" s="1"/>
-      <c r="AE16" s="1"/>
-      <c r="AF16" s="1"/>
-      <c r="AG16" s="6"/>
-      <c r="AH16" s="1"/>
-      <c r="AI16" s="1"/>
-      <c r="AK16" s="17"/>
-      <c r="AL16" s="18"/>
-      <c r="AM16" s="16"/>
-      <c r="AN16" s="17"/>
-      <c r="AO16" s="18"/>
-    </row>
-    <row r="17" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" s="1">
         <v>1530</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E17">
         <v>1583</v>
       </c>
       <c r="G17" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H17" s="1">
         <v>1478</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K17" s="1">
         <v>1223</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N17" s="1">
         <v>1098</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q17">
         <v>1336</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T17" s="1">
         <v>1303</v>
       </c>
-      <c r="V17" s="1"/>
-      <c r="W17" s="1"/>
-      <c r="Y17" s="1"/>
-      <c r="Z17" s="1"/>
-      <c r="AB17" s="1"/>
-      <c r="AC17" s="1"/>
-      <c r="AE17" s="1"/>
-      <c r="AF17" s="1"/>
-      <c r="AG17" s="6"/>
-      <c r="AH17" s="1"/>
-      <c r="AI17" s="1"/>
-      <c r="AK17" s="17"/>
-      <c r="AL17" s="18"/>
-      <c r="AM17" s="16"/>
-      <c r="AN17" s="17"/>
-      <c r="AO17" s="18"/>
-    </row>
-    <row r="18" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1">
         <v>1427</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E18">
         <v>1550</v>
       </c>
       <c r="G18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H18" s="1">
         <v>1121</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K18" s="1">
         <v>1262</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N18" s="1">
         <v>1366</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q18" s="1">
         <v>1238</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T18" s="1">
         <v>1293</v>
       </c>
-      <c r="V18" s="1"/>
-      <c r="W18" s="1"/>
-      <c r="Y18" s="1"/>
-      <c r="Z18" s="1"/>
-      <c r="AB18" s="1"/>
-      <c r="AC18" s="1"/>
-      <c r="AE18" s="1"/>
-      <c r="AF18" s="1"/>
-      <c r="AG18" s="6"/>
-      <c r="AH18" s="1"/>
-      <c r="AI18" s="1"/>
-      <c r="AK18" s="17"/>
-      <c r="AL18" s="18"/>
-      <c r="AM18" s="16"/>
-      <c r="AN18" s="17"/>
-      <c r="AO18" s="18"/>
-    </row>
-    <row r="19" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B19" s="1">
         <v>1569</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E19">
         <v>1479</v>
       </c>
       <c r="G19" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H19" s="1">
         <v>1532</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K19" s="1">
         <v>1205</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N19" s="1">
         <v>1076</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q19">
         <v>1193</v>
       </c>
       <c r="S19" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T19" s="1">
         <v>1052</v>
       </c>
-      <c r="V19" s="1"/>
-      <c r="W19" s="1"/>
-      <c r="Y19" s="1"/>
-      <c r="Z19" s="1"/>
-      <c r="AB19" s="1"/>
-      <c r="AC19" s="1"/>
-      <c r="AE19" s="1"/>
-      <c r="AF19" s="1"/>
-      <c r="AG19" s="6"/>
-      <c r="AH19" s="1"/>
-      <c r="AI19" s="1"/>
-      <c r="AK19" s="17"/>
-      <c r="AL19" s="18"/>
-      <c r="AM19" s="16"/>
-      <c r="AN19" s="17"/>
-      <c r="AO19" s="18"/>
-    </row>
-    <row r="20" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B20" s="1">
         <v>1551</v>
       </c>
       <c r="D20" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E20">
         <v>1600</v>
       </c>
       <c r="G20" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H20" s="1">
         <v>1413</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K20" s="1">
         <v>1286</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N20" s="1">
         <v>1216</v>
       </c>
       <c r="P20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q20" s="1">
         <v>1372</v>
       </c>
       <c r="S20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T20" s="1">
         <v>1325</v>
       </c>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="Y20" s="1"/>
-      <c r="Z20" s="1"/>
-      <c r="AB20" s="1"/>
-      <c r="AC20" s="1"/>
-      <c r="AE20" s="1"/>
-      <c r="AF20" s="1"/>
-      <c r="AG20" s="6"/>
-      <c r="AH20" s="1"/>
-      <c r="AI20" s="1"/>
-      <c r="AK20" s="17"/>
-      <c r="AL20" s="18"/>
-      <c r="AM20" s="16"/>
-      <c r="AN20" s="17"/>
-      <c r="AO20" s="18"/>
-    </row>
-    <row r="21" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1">
         <v>1527</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E21">
         <v>1445</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H21" s="1">
         <v>1602</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K21" s="1">
         <v>1191</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N21" s="1">
         <v>1087</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q21">
         <v>1247</v>
       </c>
       <c r="S21" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T21" s="1">
         <v>1374</v>
       </c>
-      <c r="V21" s="1"/>
-      <c r="W21" s="1"/>
-      <c r="Y21" s="1"/>
-      <c r="Z21" s="1"/>
-      <c r="AB21" s="1"/>
-      <c r="AC21" s="1"/>
-      <c r="AE21" s="1"/>
-      <c r="AF21" s="1"/>
-      <c r="AG21" s="6"/>
-      <c r="AH21" s="1"/>
-      <c r="AI21" s="1"/>
-      <c r="AK21" s="17"/>
-      <c r="AL21" s="18"/>
-      <c r="AM21" s="16"/>
-      <c r="AN21" s="17"/>
-      <c r="AO21" s="18"/>
-    </row>
-    <row r="22" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1">
         <v>1599</v>
       </c>
       <c r="D22" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E22">
         <v>1397</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H22" s="1">
         <v>1529</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K22" s="1">
         <v>1283</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N22" s="1">
         <v>1122</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q22" s="1">
         <v>1314</v>
       </c>
       <c r="S22" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T22" s="1">
         <v>1024</v>
       </c>
-      <c r="V22" s="1"/>
-      <c r="W22" s="1"/>
-      <c r="Y22" s="1"/>
-      <c r="Z22" s="1"/>
-      <c r="AB22" s="1"/>
-      <c r="AC22" s="1"/>
-      <c r="AE22" s="1"/>
-      <c r="AF22" s="1"/>
-      <c r="AG22" s="6"/>
-      <c r="AH22" s="1"/>
-      <c r="AI22" s="1"/>
-      <c r="AK22" s="17"/>
-      <c r="AL22" s="18"/>
-      <c r="AM22" s="16"/>
-      <c r="AN22" s="17"/>
-      <c r="AO22" s="18"/>
-    </row>
-    <row r="23" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1">
         <v>1533</v>
       </c>
       <c r="D23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E23">
         <v>1502</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H23" s="1">
         <v>1415</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K23" s="1">
         <v>1083</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N23" s="1">
         <v>1128</v>
       </c>
       <c r="P23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q23">
         <v>1251</v>
       </c>
       <c r="S23" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T23" s="1">
         <v>1060</v>
       </c>
-      <c r="V23" s="1"/>
-      <c r="W23" s="1"/>
-      <c r="Y23" s="1"/>
-      <c r="Z23" s="1"/>
-      <c r="AB23" s="1"/>
-      <c r="AC23" s="1"/>
-      <c r="AE23" s="1"/>
-      <c r="AF23" s="1"/>
-      <c r="AG23" s="6"/>
-      <c r="AH23" s="1"/>
-      <c r="AI23" s="1"/>
-      <c r="AK23" s="17"/>
-      <c r="AL23" s="18"/>
-      <c r="AM23" s="16"/>
-      <c r="AN23" s="17"/>
-      <c r="AO23" s="18"/>
-    </row>
-    <row r="24" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B24" s="1">
         <v>1411</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E24">
         <v>1515</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H24" s="1">
         <v>1619</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K24" s="1">
         <v>1297</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N24" s="1">
         <v>1085</v>
       </c>
       <c r="P24" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q24" s="1">
         <v>1272</v>
       </c>
       <c r="S24" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T24" s="1">
         <v>1020</v>
       </c>
-      <c r="V24" s="1"/>
-      <c r="W24" s="1"/>
-      <c r="Y24" s="1"/>
-      <c r="Z24" s="1"/>
-      <c r="AB24" s="1"/>
-      <c r="AC24" s="1"/>
-      <c r="AE24" s="1"/>
-      <c r="AF24" s="1"/>
-      <c r="AG24" s="6"/>
-      <c r="AH24" s="1"/>
-      <c r="AI24" s="1"/>
-      <c r="AK24" s="17"/>
-      <c r="AL24" s="18"/>
-      <c r="AM24" s="16"/>
-      <c r="AN24" s="17"/>
-      <c r="AO24" s="18"/>
-    </row>
-    <row r="25" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B25" s="1">
         <v>1476</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E25" s="1">
         <v>1497</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H25" s="1">
         <v>1459</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K25" s="1">
         <v>1291</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N25" s="1">
         <v>1088</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q25">
         <v>1240</v>
       </c>
       <c r="S25" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T25" s="1">
         <v>1359</v>
       </c>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AB25" s="1"/>
-      <c r="AC25" s="1"/>
-      <c r="AE25" s="1"/>
-      <c r="AF25" s="1"/>
-      <c r="AG25" s="6"/>
-      <c r="AH25" s="1"/>
-      <c r="AI25" s="1"/>
-      <c r="AK25" s="17"/>
-      <c r="AL25" s="18"/>
-      <c r="AM25" s="16"/>
-      <c r="AN25" s="17"/>
-      <c r="AO25" s="18"/>
-    </row>
-    <row r="26" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1">
         <v>1050</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E26" s="1">
         <v>1400</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H26" s="1">
         <v>1545</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K26" s="1">
         <v>1290</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N26" s="1">
         <v>1258</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q26" s="1">
         <v>1065</v>
       </c>
       <c r="S26" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T26" s="1">
         <v>1048</v>
       </c>
-      <c r="V26" s="1"/>
-      <c r="W26" s="1"/>
-      <c r="Y26" s="1"/>
-      <c r="Z26" s="1"/>
-      <c r="AB26" s="1"/>
-      <c r="AC26" s="1"/>
-      <c r="AE26" s="1"/>
-      <c r="AF26" s="1"/>
-      <c r="AG26" s="6"/>
-      <c r="AH26" s="1"/>
-      <c r="AI26" s="1"/>
-      <c r="AK26" s="17"/>
-      <c r="AL26" s="18"/>
-      <c r="AM26" s="16"/>
-      <c r="AN26" s="17"/>
-      <c r="AO26" s="18"/>
-    </row>
-    <row r="27" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B27" s="1">
         <v>1394</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E27" s="1">
         <v>1503</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H27" s="1">
         <v>1378</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K27" s="1">
         <v>1217</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N27" s="1">
         <v>1074</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q27">
         <v>1070</v>
       </c>
       <c r="S27" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T27" s="1">
         <v>1075</v>
       </c>
-      <c r="V27" s="1"/>
-      <c r="W27" s="1"/>
-      <c r="Y27" s="1"/>
-      <c r="Z27" s="1"/>
-      <c r="AB27" s="1"/>
-      <c r="AC27" s="1"/>
-      <c r="AE27" s="1"/>
-      <c r="AF27" s="1"/>
-      <c r="AG27" s="6"/>
-      <c r="AH27" s="1"/>
-      <c r="AI27" s="1"/>
-      <c r="AK27" s="17"/>
-      <c r="AL27" s="18"/>
-      <c r="AM27" s="16"/>
-      <c r="AN27" s="17"/>
-      <c r="AO27" s="18"/>
-    </row>
-    <row r="28" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B28" s="1">
         <v>1379</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E28" s="1">
         <v>1618</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H28" s="1">
         <v>1398</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K28" s="1">
         <v>1227</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N28" s="1">
         <v>1369</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q28" s="1">
         <v>1371</v>
       </c>
       <c r="S28" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T28" s="1">
         <v>1069</v>
       </c>
-      <c r="V28" s="1"/>
-      <c r="W28" s="1"/>
-      <c r="Y28" s="1"/>
-      <c r="Z28" s="1"/>
-      <c r="AB28" s="1"/>
-      <c r="AC28" s="1"/>
-      <c r="AE28" s="1"/>
-      <c r="AF28" s="1"/>
-      <c r="AG28" s="6"/>
-      <c r="AH28" s="1"/>
-      <c r="AI28" s="1"/>
-      <c r="AK28" s="17"/>
-      <c r="AL28" s="18"/>
-      <c r="AM28" s="16"/>
-      <c r="AN28" s="16"/>
-      <c r="AO28" s="16"/>
-    </row>
-    <row r="29" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B29" s="1">
         <v>1500</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E29" s="1">
         <v>1409</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H29" s="1">
         <v>1480</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K29" s="1">
         <v>1373</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N29" s="1">
         <v>1253</v>
       </c>
       <c r="P29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q29">
         <v>1334</v>
       </c>
       <c r="S29" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T29" s="1">
         <v>1058</v>
       </c>
-      <c r="V29" s="1"/>
-      <c r="W29" s="1"/>
-      <c r="Y29" s="1"/>
-      <c r="Z29" s="1"/>
-      <c r="AB29" s="1"/>
-      <c r="AC29" s="1"/>
-      <c r="AE29" s="1"/>
-      <c r="AF29" s="1"/>
-      <c r="AG29" s="6"/>
-      <c r="AH29" s="1"/>
-      <c r="AI29" s="1"/>
-      <c r="AK29" s="17"/>
-      <c r="AL29" s="18"/>
-      <c r="AM29" s="16"/>
-      <c r="AN29" s="16"/>
-      <c r="AO29" s="16"/>
-    </row>
-    <row r="30" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B30" s="1">
         <v>1392</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E30" s="1">
         <v>1542</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H30" s="1">
         <v>1534</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K30" s="1">
         <v>1295</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N30" s="1">
         <v>1237</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q30" s="1">
         <v>1367</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T30" s="1">
         <v>1059</v>
       </c>
-      <c r="V30" s="1"/>
-      <c r="W30" s="1"/>
-      <c r="Y30" s="1"/>
-      <c r="Z30" s="1"/>
-      <c r="AB30" s="1"/>
-      <c r="AC30" s="1"/>
-      <c r="AE30" s="1"/>
-      <c r="AF30" s="1"/>
-      <c r="AG30" s="6"/>
-      <c r="AH30" s="1"/>
-      <c r="AI30" s="1"/>
-      <c r="AK30" s="17"/>
-      <c r="AL30" s="18"/>
-      <c r="AM30" s="16"/>
-      <c r="AN30" s="16"/>
-      <c r="AO30" s="16"/>
-    </row>
-    <row r="31" spans="1:41" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B31" s="1">
         <v>1531</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E31" s="1">
         <v>1460</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H31" s="1">
         <v>1514</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K31" s="1">
         <v>1192</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="N31" s="1">
         <v>1312</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Q31">
         <v>1331</v>
       </c>
       <c r="S31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="T31" s="1">
         <v>1349</v>
       </c>
-      <c r="V31" s="1"/>
-      <c r="W31" s="1"/>
-      <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-      <c r="AB31" s="1"/>
-      <c r="AC31" s="1"/>
-      <c r="AE31" s="1"/>
-      <c r="AF31" s="1"/>
-      <c r="AG31" s="6"/>
-      <c r="AH31" s="1"/>
-      <c r="AI31" s="1"/>
-      <c r="AK31" s="17"/>
-      <c r="AL31" s="18"/>
-      <c r="AM31" s="16"/>
-      <c r="AN31" s="16"/>
-      <c r="AO31" s="16"/>
-    </row>
-    <row r="32" spans="1:41" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="D32" s="1"/>
@@ -2340,17 +1890,6 @@
       <c r="Q32" s="1"/>
       <c r="S32" s="1"/>
       <c r="T32" s="1"/>
-      <c r="V32" s="1"/>
-      <c r="W32" s="1"/>
-      <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-      <c r="AB32" s="1"/>
-      <c r="AC32" s="1"/>
-      <c r="AE32" s="1"/>
-      <c r="AF32" s="1"/>
-      <c r="AG32" s="6"/>
-      <c r="AH32" s="1"/>
-      <c r="AI32" s="1"/>
     </row>
     <row r="33" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
@@ -3151,11 +2690,11 @@
       <c r="A8" s="14">
         <v>5</v>
       </c>
-      <c r="B8" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>37</v>
+      <c r="B8" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>35</v>
       </c>
       <c r="D8">
         <v>321</v>

</xml_diff>